<commit_message>
v1.1.0: REF31963, Pfadkonfiguration, Bemerkungen-Default, Bereinigung
- Neues Produkt REF31963 (Sugi Instrument Wipe Xtra, 80x80mm)
- FieldDef.default_value: Felder mit Standardwert vorausfuellen (z.B. Bemerkungen = n/a)
- Messmittel + Verwendbarkeitsdatum als persistente Kontextfelder in allen Prozessen
- Bemerkungen in allen Prozessen beider Produkte, Standard n/a
- settings.py: granulare Pfade (USERS_DIR, CONFIG_DIR, PRODUCTS_DIR, AUDIT_DIR)
- Output-Dir: Produkt-Config oder Folder-Dialog, kein fester Output-Ordner mehr
- CHANGELOG.md erstellt, DOKUMENTATION.md und CLAUDE.md aktualisiert
- Version auf 1.1.0.0 angehoben
- Projektbereinigung: Planungs- und Prasentationsartefakte entfernt
- test_reader.py: Fixture nach tests/fixtures/ verschoben
</commit_message>
<xml_diff>
--- a/excel files/Vorlage_IPC4_Stanzen.xlsx
+++ b/excel files/Vorlage_IPC4_Stanzen.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Produktion\1_Artikel\1_Marke\31962\IPC_Etiketten_Packliste\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Produktion\1_Artikel\1_Marke\31963\IPC_Etiketten_Packliste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BC31068-10D3-4AD6-A9E5-BC6288AAAF1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1FD7899-69AD-4BBE-9CBD-FA6BF3A92648}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="2" r:id="rId1"/>
@@ -18,17 +18,31 @@
   </sheets>
   <externalReferences>
     <externalReference r:id="rId3"/>
+    <externalReference r:id="rId4"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Tabelle1!$A$1:$H$163</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Tabelle1!$7:$13</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="29">
   <si>
     <t>Datum</t>
   </si>
@@ -73,12 +87,6 @@
 (78 - 82 mm)</t>
   </si>
   <si>
-    <t>REF 31962</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sugi Instrument Wipe, 80x80mm, none-sterile, 250 pcs. </t>
-  </si>
-  <si>
     <t>Prüfmuster</t>
   </si>
   <si>
@@ -119,7 +127,10 @@
 (78 - 82 mm)2</t>
   </si>
   <si>
-    <t>20.01.2025 Schwehn</t>
+    <t>REF 31963</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sugi Instrument Wipe Xtra, 80x80mm, none-sterile, 250 pcs. </t>
   </si>
 </sst>
 </file>
@@ -815,15 +826,30 @@
       <sheetData sheetId="0">
         <row r="2">
           <cell r="A2" t="str">
-            <v>2030-10-31</v>
+            <v>2031-02-28</v>
           </cell>
           <cell r="B2">
-            <v>255311</v>
+            <v>265181</v>
           </cell>
         </row>
       </sheetData>
       <sheetData sheetId="1"/>
       <sheetData sheetId="2"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="IPC"/>
+      <sheetName val="Tabelle1"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1136,27 +1162,27 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J165"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="29.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="29.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.109375" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" customWidth="1"/>
     <col min="2" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="19.6640625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="19.33203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="16.6640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="21.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="19.7109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="21.28515625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
-    <row r="2" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1165,7 +1191,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:10" ht="10.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="10.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -1174,61 +1200,60 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="16">
         <f>[1]Tabelle1!$B$2</f>
-        <v>255311</v>
+        <v>265181</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="19">
-        <v>11209250</v>
-      </c>
-      <c r="G4" s="30" t="s">
-        <v>29</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F4" s="19"/>
+      <c r="G4" s="30"/>
       <c r="H4" s="18"/>
     </row>
-    <row r="5" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="17" t="str">
         <f>[1]Tabelle1!$A$2</f>
-        <v>2030-10-31</v>
+        <v>2031-02-28</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E5" s="33">
         <v>60000</v>
       </c>
       <c r="F5" s="34" t="s">
-        <v>23</v>
-      </c>
-      <c r="G5" s="39"/>
+        <v>21</v>
+      </c>
+      <c r="G5" s="39" t="e">
+        <f>IF(E5&gt;=[2]Tabelle1!#REF!,[2]Tabelle1!B17,IF(E5&gt;=[2]Tabelle1!#REF!,[2]Tabelle1!B16,IF(E5&gt;=[2]Tabelle1!#REF!,[2]Tabelle1!B15,IF(E5&gt;=[2]Tabelle1!#REF!,[2]Tabelle1!B14,IF(E5&gt;=[2]Tabelle1!#REF!,[2]Tabelle1!B13,IF(E5&gt;=[2]Tabelle1!#REF!,[2]Tabelle1!B12,IF(E5&gt;=[2]Tabelle1!#REF!,[2]Tabelle1!B11,IF(E5&gt;=[2]Tabelle1!#REF!,[2]Tabelle1!B10,IF(E5&gt;=[2]Tabelle1!#REF!,[2]Tabelle1!B9,IF(E5&gt;=[2]Tabelle1!#REF!,[2]Tabelle1!B8,IF(E5&gt;=[2]Tabelle1!#REF!,[2]Tabelle1!B7,IF(E5&gt;=[2]Tabelle1!#REF!,[2]Tabelle1!B6,IF(E5&gt;=[2]Tabelle1!#REF!,[2]Tabelle1!B5,IF(E5&gt;=[2]Tabelle1!#REF!,[2]Tabelle1!B4,IF(E5&gt;=[2]Tabelle1!#REF!,[2]Tabelle1!B3,IF(E5&gt;=[2]Tabelle1!#REF!,[2]Tabelle1!B2))))))))))))))))</f>
+        <v>#REF!</v>
+      </c>
       <c r="H5" s="35" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D6" s="36">
         <f>E5*1</f>
         <v>60000</v>
       </c>
       <c r="F6" s="37" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G6" s="38"/>
     </row>
-    <row r="7" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -1239,14 +1264,14 @@
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="1:10" ht="10.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" ht="10.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>8</v>
       </c>
@@ -1263,7 +1288,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>8</v>
       </c>
@@ -1282,7 +1307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>8</v>
       </c>
@@ -1301,7 +1326,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="21" t="s">
         <v>8</v>
       </c>
@@ -1320,21 +1345,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="25" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B13" s="26" t="s">
         <v>12</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D13" s="26" t="s">
         <v>13</v>
       </c>
       <c r="E13" s="26" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F13" s="26" t="s">
         <v>0</v>
@@ -1346,7 +1371,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="13"/>
       <c r="B14" s="31"/>
       <c r="C14" s="29">
@@ -1361,7 +1386,7 @@
       </c>
       <c r="J14" s="40"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>
       <c r="B15" s="31"/>
       <c r="C15" s="29">
@@ -1376,7 +1401,7 @@
       </c>
       <c r="J15" s="40"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="13"/>
       <c r="B16" s="31"/>
       <c r="C16" s="29">
@@ -1391,7 +1416,7 @@
       </c>
       <c r="J16" s="40"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="13"/>
       <c r="B17" s="31"/>
       <c r="C17" s="29">
@@ -1406,7 +1431,7 @@
       </c>
       <c r="J17" s="40"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="13"/>
       <c r="B18" s="31"/>
       <c r="C18" s="29">
@@ -1420,7 +1445,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="13"/>
       <c r="B19" s="31"/>
       <c r="C19" s="29">
@@ -1434,7 +1459,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="13"/>
       <c r="B20" s="31"/>
       <c r="C20" s="29">
@@ -1448,7 +1473,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="13"/>
       <c r="B21" s="31"/>
       <c r="C21" s="29">
@@ -1462,7 +1487,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="13"/>
       <c r="B22" s="31"/>
       <c r="C22" s="29">
@@ -1476,7 +1501,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="13"/>
       <c r="B23" s="31"/>
       <c r="C23" s="29">
@@ -1490,7 +1515,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="13"/>
       <c r="B24" s="31"/>
       <c r="C24" s="29">
@@ -1504,7 +1529,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="13"/>
       <c r="B25" s="31"/>
       <c r="C25" s="29">
@@ -1518,7 +1543,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="13"/>
       <c r="B26" s="31"/>
       <c r="C26" s="29">
@@ -1532,7 +1557,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="13"/>
       <c r="B27" s="31"/>
       <c r="C27" s="29">
@@ -1546,7 +1571,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="13"/>
       <c r="B28" s="31"/>
       <c r="C28" s="29">
@@ -1560,7 +1585,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="13"/>
       <c r="B29" s="31"/>
       <c r="C29" s="29">
@@ -1574,7 +1599,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="13"/>
       <c r="B30" s="31"/>
       <c r="C30" s="29">
@@ -1588,7 +1613,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="13"/>
       <c r="B31" s="31"/>
       <c r="C31" s="29">
@@ -1602,7 +1627,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="13"/>
       <c r="B32" s="31"/>
       <c r="C32" s="29">
@@ -1616,7 +1641,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="13"/>
       <c r="B33" s="31"/>
       <c r="C33" s="29">
@@ -1630,7 +1655,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="13"/>
       <c r="B34" s="31"/>
       <c r="C34" s="29">
@@ -1644,7 +1669,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="13"/>
       <c r="B35" s="31"/>
       <c r="C35" s="29">
@@ -1658,7 +1683,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="13"/>
       <c r="B36" s="31"/>
       <c r="C36" s="29">
@@ -1672,7 +1697,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="13"/>
       <c r="B37" s="31"/>
       <c r="C37" s="29">
@@ -1686,7 +1711,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="13"/>
       <c r="B38" s="31"/>
       <c r="C38" s="29">
@@ -1700,7 +1725,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="13"/>
       <c r="B39" s="31"/>
       <c r="C39" s="29">
@@ -1714,7 +1739,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="13"/>
       <c r="B40" s="31"/>
       <c r="C40" s="29">
@@ -1728,7 +1753,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="13"/>
       <c r="B41" s="31"/>
       <c r="C41" s="29">
@@ -1742,7 +1767,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="13"/>
       <c r="B42" s="31"/>
       <c r="C42" s="29">
@@ -1756,7 +1781,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="13"/>
       <c r="B43" s="31"/>
       <c r="C43" s="29">
@@ -1770,7 +1795,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="13"/>
       <c r="B44" s="31"/>
       <c r="C44" s="29">
@@ -1784,7 +1809,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="13"/>
       <c r="B45" s="31"/>
       <c r="C45" s="29">
@@ -1798,7 +1823,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="13"/>
       <c r="B46" s="31"/>
       <c r="C46" s="29">
@@ -1812,7 +1837,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="13"/>
       <c r="B47" s="31"/>
       <c r="C47" s="29">
@@ -1826,7 +1851,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="13"/>
       <c r="B48" s="31"/>
       <c r="C48" s="29">
@@ -1840,7 +1865,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="13"/>
       <c r="B49" s="31"/>
       <c r="C49" s="29">
@@ -1854,7 +1879,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="13"/>
       <c r="B50" s="31"/>
       <c r="C50" s="29">
@@ -1868,7 +1893,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="13"/>
       <c r="B51" s="31"/>
       <c r="C51" s="29">
@@ -1882,7 +1907,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="13"/>
       <c r="B52" s="31"/>
       <c r="C52" s="29">
@@ -1896,7 +1921,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="13"/>
       <c r="B53" s="31"/>
       <c r="C53" s="29">
@@ -1910,7 +1935,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="13"/>
       <c r="B54" s="31"/>
       <c r="C54" s="29">
@@ -1924,7 +1949,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="13"/>
       <c r="B55" s="31"/>
       <c r="C55" s="29">
@@ -1938,7 +1963,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="13"/>
       <c r="B56" s="31"/>
       <c r="C56" s="29">
@@ -1952,7 +1977,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="13"/>
       <c r="B57" s="31"/>
       <c r="C57" s="29">
@@ -1966,7 +1991,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="13"/>
       <c r="B58" s="31"/>
       <c r="C58" s="29">
@@ -1980,7 +2005,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="13"/>
       <c r="B59" s="31"/>
       <c r="C59" s="29">
@@ -1994,7 +2019,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="13"/>
       <c r="B60" s="31"/>
       <c r="C60" s="29">
@@ -2008,7 +2033,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="13"/>
       <c r="B61" s="31"/>
       <c r="C61" s="29">
@@ -2022,7 +2047,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="13"/>
       <c r="B62" s="31"/>
       <c r="C62" s="29">
@@ -2036,7 +2061,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="13"/>
       <c r="B63" s="31"/>
       <c r="C63" s="29">
@@ -2050,7 +2075,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="13"/>
       <c r="B64" s="31"/>
       <c r="C64" s="29">
@@ -2064,7 +2089,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="13"/>
       <c r="B65" s="31"/>
       <c r="C65" s="29">
@@ -2078,7 +2103,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="13"/>
       <c r="B66" s="31"/>
       <c r="C66" s="29">
@@ -2092,7 +2117,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="13"/>
       <c r="B67" s="31"/>
       <c r="C67" s="29">
@@ -2106,7 +2131,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="13"/>
       <c r="B68" s="31"/>
       <c r="C68" s="29">
@@ -2120,7 +2145,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="13"/>
       <c r="B69" s="31"/>
       <c r="C69" s="29">
@@ -2134,7 +2159,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="13"/>
       <c r="B70" s="31"/>
       <c r="C70" s="29">
@@ -2148,7 +2173,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="13"/>
       <c r="B71" s="31"/>
       <c r="C71" s="29">
@@ -2162,7 +2187,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="13"/>
       <c r="B72" s="31"/>
       <c r="C72" s="29">
@@ -2176,7 +2201,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="13"/>
       <c r="B73" s="31"/>
       <c r="C73" s="29">
@@ -2190,7 +2215,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="13"/>
       <c r="B74" s="31"/>
       <c r="C74" s="29">
@@ -2204,7 +2229,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" s="13"/>
       <c r="B75" s="31"/>
       <c r="C75" s="29">
@@ -2218,7 +2243,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" s="13"/>
       <c r="B76" s="31"/>
       <c r="C76" s="29">
@@ -2232,7 +2257,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" s="13"/>
       <c r="B77" s="31"/>
       <c r="C77" s="29">
@@ -2246,7 +2271,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" s="13"/>
       <c r="B78" s="31"/>
       <c r="C78" s="29">
@@ -2260,7 +2285,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" s="13"/>
       <c r="B79" s="31"/>
       <c r="C79" s="29">
@@ -2274,7 +2299,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" s="13"/>
       <c r="B80" s="31"/>
       <c r="C80" s="29">
@@ -2288,7 +2313,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="13"/>
       <c r="B81" s="31"/>
       <c r="C81" s="29">
@@ -2302,7 +2327,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="13"/>
       <c r="B82" s="31"/>
       <c r="C82" s="29">
@@ -2316,7 +2341,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" s="13"/>
       <c r="B83" s="31"/>
       <c r="C83" s="29">
@@ -2330,7 +2355,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" s="13"/>
       <c r="B84" s="31"/>
       <c r="C84" s="29">
@@ -2344,7 +2369,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" s="13"/>
       <c r="B85" s="31"/>
       <c r="C85" s="29">
@@ -2358,7 +2383,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" s="13"/>
       <c r="B86" s="31"/>
       <c r="C86" s="29">
@@ -2372,7 +2397,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" s="13"/>
       <c r="B87" s="31"/>
       <c r="C87" s="29">
@@ -2386,7 +2411,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" s="13"/>
       <c r="B88" s="31"/>
       <c r="C88" s="29">
@@ -2400,7 +2425,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" s="13"/>
       <c r="B89" s="31"/>
       <c r="C89" s="29">
@@ -2414,7 +2439,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" s="13"/>
       <c r="B90" s="31"/>
       <c r="C90" s="29">
@@ -2428,7 +2453,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" s="13"/>
       <c r="B91" s="31"/>
       <c r="C91" s="29">
@@ -2442,7 +2467,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" s="13"/>
       <c r="B92" s="31"/>
       <c r="C92" s="29">
@@ -2456,7 +2481,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" s="13"/>
       <c r="B93" s="31"/>
       <c r="C93" s="29">
@@ -2470,7 +2495,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" s="13"/>
       <c r="B94" s="31"/>
       <c r="C94" s="29">
@@ -2484,7 +2509,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" s="13"/>
       <c r="B95" s="31"/>
       <c r="C95" s="29">
@@ -2498,7 +2523,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" s="13"/>
       <c r="B96" s="31"/>
       <c r="C96" s="29">
@@ -2512,7 +2537,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" s="13"/>
       <c r="B97" s="31"/>
       <c r="C97" s="29">
@@ -2526,7 +2551,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" s="13"/>
       <c r="B98" s="31"/>
       <c r="C98" s="29">
@@ -2540,7 +2565,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" s="13"/>
       <c r="B99" s="31"/>
       <c r="C99" s="29">
@@ -2554,7 +2579,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" s="13"/>
       <c r="B100" s="31"/>
       <c r="C100" s="29">
@@ -2568,7 +2593,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" s="13"/>
       <c r="B101" s="31"/>
       <c r="C101" s="29">
@@ -2582,7 +2607,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" s="13"/>
       <c r="B102" s="31"/>
       <c r="C102" s="29">
@@ -2596,7 +2621,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" s="13"/>
       <c r="B103" s="31"/>
       <c r="C103" s="29">
@@ -2610,7 +2635,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" s="13"/>
       <c r="B104" s="31"/>
       <c r="C104" s="29">
@@ -2624,7 +2649,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" s="13"/>
       <c r="B105" s="31"/>
       <c r="C105" s="29">
@@ -2638,7 +2663,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" s="13"/>
       <c r="B106" s="31"/>
       <c r="C106" s="29">
@@ -2652,7 +2677,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" s="13"/>
       <c r="B107" s="31"/>
       <c r="C107" s="29">
@@ -2666,7 +2691,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" s="13"/>
       <c r="B108" s="31"/>
       <c r="C108" s="29">
@@ -2680,7 +2705,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" s="13"/>
       <c r="B109" s="31"/>
       <c r="C109" s="29">
@@ -2694,7 +2719,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" s="13"/>
       <c r="B110" s="31"/>
       <c r="C110" s="29">
@@ -2708,7 +2733,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" s="13"/>
       <c r="B111" s="31"/>
       <c r="C111" s="29">
@@ -2722,7 +2747,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" s="13"/>
       <c r="B112" s="31"/>
       <c r="C112" s="29">
@@ -2736,7 +2761,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113" s="13"/>
       <c r="B113" s="31"/>
       <c r="C113" s="29">
@@ -2750,7 +2775,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114" s="13"/>
       <c r="B114" s="31"/>
       <c r="C114" s="29">
@@ -2764,7 +2789,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115" s="13"/>
       <c r="B115" s="31"/>
       <c r="C115" s="29">
@@ -2778,7 +2803,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" s="13"/>
       <c r="B116" s="31"/>
       <c r="C116" s="29">
@@ -2792,7 +2817,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117" s="13"/>
       <c r="B117" s="31"/>
       <c r="C117" s="29">
@@ -2806,7 +2831,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118" s="13"/>
       <c r="B118" s="31"/>
       <c r="C118" s="29">
@@ -2820,7 +2845,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119" s="13"/>
       <c r="B119" s="31"/>
       <c r="C119" s="29">
@@ -2834,7 +2859,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120" s="13"/>
       <c r="B120" s="31"/>
       <c r="C120" s="29">
@@ -2848,7 +2873,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A121" s="13"/>
       <c r="B121" s="31"/>
       <c r="C121" s="29">
@@ -2862,7 +2887,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122" s="13"/>
       <c r="B122" s="31"/>
       <c r="C122" s="29">
@@ -2876,7 +2901,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123" s="13"/>
       <c r="B123" s="31"/>
       <c r="C123" s="29">
@@ -2890,7 +2915,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124" s="13"/>
       <c r="B124" s="31"/>
       <c r="C124" s="29">
@@ -2904,7 +2929,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A125" s="13"/>
       <c r="B125" s="31"/>
       <c r="C125" s="29">
@@ -2918,7 +2943,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126" s="13"/>
       <c r="B126" s="31"/>
       <c r="C126" s="29">
@@ -2932,7 +2957,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127" s="13"/>
       <c r="B127" s="31"/>
       <c r="C127" s="29">
@@ -2946,7 +2971,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A128" s="13"/>
       <c r="B128" s="31"/>
       <c r="C128" s="29">
@@ -2960,7 +2985,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A129" s="13"/>
       <c r="B129" s="31"/>
       <c r="C129" s="29">
@@ -2974,7 +2999,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A130" s="13"/>
       <c r="B130" s="31"/>
       <c r="C130" s="29">
@@ -2988,7 +3013,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A131" s="13"/>
       <c r="B131" s="31"/>
       <c r="C131" s="29">
@@ -3002,7 +3027,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A132" s="13"/>
       <c r="B132" s="31"/>
       <c r="C132" s="29">
@@ -3016,7 +3041,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A133" s="13"/>
       <c r="B133" s="31"/>
       <c r="C133" s="29">
@@ -3030,7 +3055,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A134" s="13"/>
       <c r="B134" s="31"/>
       <c r="C134" s="29">
@@ -3044,7 +3069,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A135" s="13"/>
       <c r="B135" s="31"/>
       <c r="C135" s="29">
@@ -3058,7 +3083,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A136" s="13"/>
       <c r="B136" s="31"/>
       <c r="C136" s="29">
@@ -3072,7 +3097,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A137" s="13"/>
       <c r="B137" s="31"/>
       <c r="C137" s="29">
@@ -3086,7 +3111,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A138" s="13"/>
       <c r="B138" s="31"/>
       <c r="C138" s="29">
@@ -3100,7 +3125,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A139" s="13"/>
       <c r="B139" s="31"/>
       <c r="C139" s="29">
@@ -3114,7 +3139,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A140" s="13"/>
       <c r="B140" s="31"/>
       <c r="C140" s="29">
@@ -3128,7 +3153,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A141" s="13"/>
       <c r="B141" s="31"/>
       <c r="C141" s="29">
@@ -3142,7 +3167,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A142" s="13"/>
       <c r="B142" s="31"/>
       <c r="C142" s="29">
@@ -3156,7 +3181,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A143" s="13"/>
       <c r="B143" s="31"/>
       <c r="C143" s="29">
@@ -3170,7 +3195,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A144" s="13"/>
       <c r="B144" s="31"/>
       <c r="C144" s="29">
@@ -3184,7 +3209,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A145" s="13"/>
       <c r="B145" s="31"/>
       <c r="C145" s="29">
@@ -3198,7 +3223,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A146" s="13"/>
       <c r="B146" s="31"/>
       <c r="C146" s="29">
@@ -3212,7 +3237,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A147" s="13"/>
       <c r="B147" s="31"/>
       <c r="C147" s="29">
@@ -3226,7 +3251,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A148" s="13"/>
       <c r="B148" s="31"/>
       <c r="C148" s="29">
@@ -3240,7 +3265,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A149" s="13"/>
       <c r="B149" s="31"/>
       <c r="C149" s="29">
@@ -3254,7 +3279,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A150" s="13"/>
       <c r="B150" s="31"/>
       <c r="C150" s="29">
@@ -3268,7 +3293,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A151" s="13"/>
       <c r="B151" s="31"/>
       <c r="C151" s="29">
@@ -3282,7 +3307,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A152" s="13"/>
       <c r="B152" s="31"/>
       <c r="C152" s="29">
@@ -3296,7 +3321,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A153" s="13"/>
       <c r="B153" s="31"/>
       <c r="C153" s="29">
@@ -3310,7 +3335,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A154" s="13"/>
       <c r="B154" s="31"/>
       <c r="C154" s="29">
@@ -3324,7 +3349,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A155" s="13"/>
       <c r="B155" s="31"/>
       <c r="C155" s="29">
@@ -3338,7 +3363,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A156" s="13"/>
       <c r="B156" s="31"/>
       <c r="C156" s="29">
@@ -3352,7 +3377,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A157" s="13"/>
       <c r="B157" s="31"/>
       <c r="C157" s="29">
@@ -3366,7 +3391,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A158" s="13"/>
       <c r="B158" s="31"/>
       <c r="C158" s="29">
@@ -3380,7 +3405,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A159" s="13"/>
       <c r="B159" s="31"/>
       <c r="C159" s="29">
@@ -3394,7 +3419,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A160" s="13"/>
       <c r="B160" s="31"/>
       <c r="C160" s="29">
@@ -3408,7 +3433,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A161" s="13"/>
       <c r="B161" s="31"/>
       <c r="C161" s="29">
@@ -3422,7 +3447,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="162" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A162" s="13"/>
       <c r="B162" s="31"/>
       <c r="C162" s="29">
@@ -3436,7 +3461,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="163" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A163" s="13"/>
       <c r="B163" s="31"/>
       <c r="C163" s="29">
@@ -3450,13 +3475,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="165" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="B0qf4rTPaDfrEN3i/McHZDgGo3utdnZdDnoNE9qPgBzjLnZ/Tds2A164cZTM17qu+W/Wjid4sFPrkfj0fEQbmw==" saltValue="ivxt4Y8ufUiGiNMtFfXhAA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
     <mergeCell ref="J14:J17"/>
   </mergeCells>
@@ -3501,22 +3525,22 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7071106-8BC5-4671-A414-ED9B4A637616}">
   <dimension ref="A1:C18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="B1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3527,7 +3551,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>9</v>
       </c>
@@ -3538,7 +3562,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>16</v>
       </c>
@@ -3549,7 +3573,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>26</v>
       </c>
@@ -3560,7 +3584,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>51</v>
       </c>
@@ -3571,7 +3595,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>91</v>
       </c>
@@ -3582,7 +3606,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>151</v>
       </c>
@@ -3593,7 +3617,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>281</v>
       </c>
@@ -3604,7 +3628,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>401</v>
       </c>
@@ -3615,7 +3639,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>501</v>
       </c>
@@ -3626,7 +3650,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1201</v>
       </c>
@@ -3637,7 +3661,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>3201</v>
       </c>
@@ -3648,7 +3672,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>10001</v>
       </c>
@@ -3659,7 +3683,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>35001</v>
       </c>
@@ -3670,7 +3694,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>150001</v>
       </c>
@@ -3681,12 +3705,12 @@
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>500001</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C18">
         <v>150</v>

</xml_diff>